<commit_message>
Stage 8 fixes: B-024
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2021/BW21_0240/Run_sheets/BW21_0240_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2021/BW21_0240/Run_sheets/BW21_0240_RUN04.xlsx
@@ -188,21 +188,6 @@
 </file>
 
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Stéphane Guillaume</author>
-  </authors>
-  <commentList>
-    <comment ref="H4" authorId="0" shapeId="0">
-      <text>
-        <t>Re-dispense on PA-13 was a pipetting correction before read, not a re-run. Noted here for the record.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Ravi Deshmukh</author>
@@ -659,7 +644,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Primary IC50, first 12 compounds</t>
+          <t>Interim membership: original dated run records; no inferred first-twelve subset</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -738,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -754,235 +739,98 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Plate</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Compound block</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Top conc</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Reference inhibitor</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Vehicle</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
+          <t>Plate assignment and control acceptance: source-record index</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PA-11</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Interim</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>TP04-02701 to 02712</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>10 µM</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Read after the Z' check</t>
+          <t>Use</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PA-12</t>
+          <t>Full primary inventory</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>Every compound on Primary IC50</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>TP04-02713 to 02724</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>10 µM</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>All reported IDs, including those after TP04-02748, belong to the inventory; consecutive ranges are not plate assignments.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PA-13</t>
+          <t>Compound-to-plate mapping</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>BW21_0240 original RUN04 layouts and sample cards under B-ACC-2021-04086</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>TP04-02725 to 02736</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>10 µM</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Two wells re-dispensed</t>
+          <t>Use plate/well field for each compound; mapping is not reproduced here.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PA-14</t>
+          <t>Interim membership</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>27/07/2021 run records linked to sample cards</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>TP04-02737 to 02748</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>10 µM</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Within range</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6"/>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Acceptance as per study plan. Reference inhibitor and vehicle both within the historical range on every plate; the selectivity plates were read against the same reference.</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Plate acceptance: all four plates accepted for the final fit.</t>
+          <t>No interim membership inferred from ID order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Control validity</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Original plate acceptance records and study-plan criteria</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>No per-plate acceptance result asserted by this index.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A6:H6"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1011,7 +859,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hill slopes outside the study plan window were re-fitted with the top fixed before the value was accepted. Replicate fits are on the run sheet.</t>
+          <t>One summary IC50 and Hill slope per compound are shown. Replicate curves, fit settings and plate/well mapping are not reproduced; no top-fixed rescue rule or affected-compound list asserted. Consult original RUN04 curve records linked to sample cards under B-ACC-2021-04086 for processing history.</t>
         </is>
       </c>
     </row>

</xml_diff>